<commit_message>
enhanced the ui and other features
</commit_message>
<xml_diff>
--- a/users/ck/Sandhata_Internship_Log.xlsx
+++ b/users/ck/Sandhata_Internship_Log.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,12 @@
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -63,8 +67,14 @@
         <bgColor rgb="00DCE6F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -86,11 +96,88 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -102,6 +189,25 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -488,13 +594,13 @@
           <t>SANDHATA INTERNSHIP</t>
         </is>
       </c>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="5" t="n"/>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="5" t="n"/>
+      <c r="H1" s="5" t="n"/>
+      <c r="I1" s="5" t="n"/>
+      <c r="J1" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -510,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -529,13 +635,13 @@
           <t>SANDHATA INTERNSHIP - TIMESHEET LOG</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="5" t="n"/>
+      <c r="C1" s="5" t="n"/>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="5" t="n"/>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="5" t="n"/>
+      <c r="H1" s="6" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
@@ -579,8 +685,286 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>WEEK 2</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>DAY 5</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>12/06/2026</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n"/>
+      <c r="B4" s="12" t="n"/>
+      <c r="C4" s="12" t="n"/>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n"/>
+      <c r="B5" s="12" t="n"/>
+      <c r="C5" s="12" t="n"/>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="n"/>
+      <c r="B7" s="13" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>WEEK 2</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>DAY 2</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>12/06/2026</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n"/>
+      <c r="B10" s="9" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n"/>
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="7">
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="C8:C12"/>
+    <mergeCell ref="C3:C7"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B3:B7"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added Toggle button to sidebar
</commit_message>
<xml_diff>
--- a/users/ck/Sandhata_Internship_Log.xlsx
+++ b/users/ck/Sandhata_Internship_Log.xlsx
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -858,9 +858,9 @@
       <c r="H8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n"/>
-      <c r="B9" s="1" t="n"/>
-      <c r="C9" s="7" t="n"/>
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
       <c r="D9" s="7" t="inlineStr">
         <is>
           <t>11:00</t>
@@ -882,9 +882,9 @@
       <c r="H9" s="8" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="n"/>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="10" t="n"/>
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
       <c r="D10" s="10" t="inlineStr">
         <is>
           <t>13:00</t>
@@ -910,9 +910,9 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n"/>
-      <c r="B11" s="1" t="n"/>
-      <c r="C11" s="7" t="n"/>
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
       <c r="D11" s="7" t="inlineStr">
         <is>
           <t>14:00</t>
@@ -934,9 +934,9 @@
       <c r="H11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n"/>
-      <c r="B12" s="1" t="n"/>
-      <c r="C12" s="7" t="n"/>
+      <c r="A12" s="13" t="n"/>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
       <c r="D12" s="7" t="inlineStr">
         <is>
           <t>16:00</t>
@@ -957,14 +957,153 @@
       </c>
       <c r="H12" s="8" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>WEEK 3</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>DAY 1</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>15/06/2026</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n"/>
+      <c r="B14" s="1" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n"/>
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="1" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n"/>
+      <c r="B17" s="1" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="10">
+    <mergeCell ref="C13:C17"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="C8:C12"/>
+    <mergeCell ref="B13:B17"/>
     <mergeCell ref="C3:C7"/>
     <mergeCell ref="A3:A7"/>
     <mergeCell ref="B3:B7"/>
+    <mergeCell ref="A13:A17"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fixed sidebar bugs and darkmode bugs
</commit_message>
<xml_diff>
--- a/users/ck/Sandhata_Internship_Log.xlsx
+++ b/users/ck/Sandhata_Internship_Log.xlsx
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -994,9 +994,9 @@
       <c r="H13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n"/>
-      <c r="B14" s="1" t="n"/>
-      <c r="C14" s="7" t="n"/>
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
       <c r="D14" s="7" t="inlineStr">
         <is>
           <t>11:00</t>
@@ -1018,9 +1018,9 @@
       <c r="H14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="n"/>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="10" t="n"/>
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
       <c r="D15" s="10" t="inlineStr">
         <is>
           <t>13:00</t>
@@ -1046,9 +1046,9 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n"/>
-      <c r="B16" s="1" t="n"/>
-      <c r="C16" s="7" t="n"/>
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="12" t="n"/>
       <c r="D16" s="7" t="inlineStr">
         <is>
           <t>14:00</t>
@@ -1070,9 +1070,9 @@
       <c r="H16" s="8" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n"/>
-      <c r="B17" s="1" t="n"/>
-      <c r="C17" s="7" t="n"/>
+      <c r="A17" s="13" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="n"/>
       <c r="D17" s="7" t="inlineStr">
         <is>
           <t>16:00</t>
@@ -1093,8 +1093,287 @@
       </c>
       <c r="H17" s="8" t="inlineStr"/>
     </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>WEEK 1</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>DAY 1</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>15/06/2026</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n"/>
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="n"/>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>WEEK 2</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>DAY 1</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>15/06/2026</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n"/>
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n"/>
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t>Lunch Break</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n"/>
+      <c r="B26" s="12" t="n"/>
+      <c r="C26" s="12" t="n"/>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Completed the scrum meeting, given all the updates. And testing our project prototype.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="n"/>
+      <c r="B27" s="13" t="n"/>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="16">
+    <mergeCell ref="C18:C22"/>
+    <mergeCell ref="A18:A22"/>
+    <mergeCell ref="B18:B22"/>
     <mergeCell ref="C13:C17"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="B8:B12"/>
@@ -1105,6 +1384,9 @@
     <mergeCell ref="B3:B7"/>
     <mergeCell ref="A13:A17"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B23:B27"/>
+    <mergeCell ref="C23:C27"/>
+    <mergeCell ref="A23:A27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>